<commit_message>
Updated metrics and metrics pdf
</commit_message>
<xml_diff>
--- a/sprint6/26-04-sprint-6-metrics.xlsx
+++ b/sprint6/26-04-sprint-6-metrics.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\styne\Lewis\1-Spring26\software\sprint6\Stone-Ocean-Backlogs\sprint6\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13000CD2-F357-445C-945B-6CA818C6AAC6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D994B3D5-55EF-45AA-8EF4-EF6C9FAB2159}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="9876" yWindow="1128" windowWidth="11472" windowHeight="10776" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37134,7 +37134,7 @@
         <v>6</v>
       </c>
       <c r="C9" s="7">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D9" s="7">
         <v>0</v>
@@ -37224,7 +37224,7 @@
         <v>6</v>
       </c>
       <c r="C12" s="7">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D12" s="7">
         <v>0</v>
@@ -37289,7 +37289,7 @@
       </c>
       <c r="C16" s="7">
         <f>SUM(C9:C14)</f>
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="D16" s="7">
         <f>SUM(D9:D14)</f>

</xml_diff>

<commit_message>
Update sprint6 backlog and created final versions for backlog and metrics
</commit_message>
<xml_diff>
--- a/sprint6/26-04-sprint-6-metrics.xlsx
+++ b/sprint6/26-04-sprint-6-metrics.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\styne\Lewis\1-Spring26\software\sprint6\Stone-Ocean-Backlogs\sprint6\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A5691872-E695-4098-B39E-8E39BF7459A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1705A79-8256-48F6-B7EC-96C7603ED221}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="9876" yWindow="1128" windowWidth="11472" windowHeight="10776" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="8568" yWindow="1308" windowWidth="11472" windowHeight="10776" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Example" sheetId="8" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="212" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="216" uniqueCount="45">
   <si>
     <t>Name</t>
   </si>
@@ -170,6 +170,12 @@
   </si>
   <si>
     <t>April 14th, 2026; 10:10am</t>
+  </si>
+  <si>
+    <t>April 26th, 2026; 8:46pm</t>
+  </si>
+  <si>
+    <t>April 26th, 2026; 8:52pm</t>
   </si>
 </sst>
 </file>
@@ -37137,23 +37143,23 @@
         <v>7</v>
       </c>
       <c r="D9" s="7">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="E9" s="7">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F9" s="8"/>
       <c r="G9" s="9">
         <f t="shared" ref="G9:H12" si="0">D9/B9</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H9" s="10">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.5714285714285714</v>
       </c>
       <c r="I9" s="10">
         <f t="shared" ref="I9:I16" si="1">E9/B9</f>
-        <v>0</v>
+        <v>0.66666666666666663</v>
       </c>
     </row>
     <row r="10" spans="1:9" ht="15.75" customHeight="1">
@@ -37167,23 +37173,23 @@
         <v>7</v>
       </c>
       <c r="D10" s="7">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="E10" s="7">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="F10" s="8"/>
       <c r="G10" s="9">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>1.1666666666666667</v>
       </c>
       <c r="H10" s="10">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I10" s="10">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>1.1666666666666667</v>
       </c>
     </row>
     <row r="11" spans="1:9" ht="15.75" customHeight="1">
@@ -37197,23 +37203,23 @@
         <v>6</v>
       </c>
       <c r="D11" s="7">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="E11" s="7">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F11" s="8"/>
       <c r="G11" s="9">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.83333333333333337</v>
       </c>
       <c r="H11" s="10">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="I11" s="10">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="12" spans="1:9" ht="15.75" customHeight="1">
@@ -37227,23 +37233,23 @@
         <v>6</v>
       </c>
       <c r="D12" s="7">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="E12" s="7">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="F12" s="8"/>
       <c r="G12" s="9">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H12" s="10">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I12" s="10">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="13" spans="1:9" ht="15.75" customHeight="1">
@@ -37293,24 +37299,24 @@
       </c>
       <c r="D16" s="7">
         <f>SUM(D9:D14)</f>
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="E16" s="7">
         <f>SUM(E9:E14)</f>
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="F16" s="8"/>
       <c r="G16" s="9">
         <f t="shared" ref="G16:H16" si="2">D16/B16</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H16" s="10">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>0.76923076923076927</v>
       </c>
       <c r="I16" s="10">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>0.83333333333333337</v>
       </c>
     </row>
     <row r="17" spans="1:9" ht="15.75" customHeight="1">
@@ -37387,18 +37393,26 @@
       <c r="A24" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="B24" s="16"/>
+      <c r="B24" s="16" t="s">
+        <v>39</v>
+      </c>
       <c r="C24" s="16"/>
-      <c r="D24" s="17"/>
+      <c r="D24" s="17" t="s">
+        <v>43</v>
+      </c>
       <c r="E24" s="3"/>
     </row>
     <row r="25" spans="1:9" ht="15.75" customHeight="1">
       <c r="A25" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="B25" s="10"/>
+      <c r="B25" s="10" t="s">
+        <v>41</v>
+      </c>
       <c r="C25" s="16"/>
-      <c r="D25" s="17"/>
+      <c r="D25" s="17" t="s">
+        <v>44</v>
+      </c>
       <c r="E25" s="7"/>
     </row>
     <row r="26" spans="1:9" ht="15.75" customHeight="1">

</xml_diff>